<commit_message>
Add cache-busting parameter for template download
Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A4FEA1-1F43-4D61-9F63-6B8ECC7EE9DA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA8766C7-E70B-4E6E-B769-659503E2796D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9648" tabRatio="639" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9648" tabRatio="639" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="x월 하자보수비 금액" sheetId="82" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5268" uniqueCount="1115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5269" uniqueCount="1116">
   <si>
     <t>판정형태</t>
   </si>
@@ -4334,6 +4334,10 @@
   <si>
     <t>성채은</t>
   </si>
+  <si>
+    <t>당월 매출</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -4343,7 +4347,7 @@
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="176" formatCode="#,##0_ "/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -4401,6 +4405,12 @@
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="9">
@@ -4556,7 +4566,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4679,6 +4689,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="쉼표 [0] 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -5067,10 +5081,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{740B8B6B-1FF8-46A0-911F-F1F62C78BC45}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="9" max="9" width="12.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.35">
       <c r="A1" s="45" t="s">
         <v>27</v>
       </c>
@@ -5095,8 +5112,11 @@
       <c r="H1" s="45" t="s">
         <v>8</v>
       </c>
+      <c r="I1" s="46" t="s">
+        <v>1115</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="45" t="s">
         <v>6</v>
       </c>
@@ -5120,6 +5140,9 @@
       </c>
       <c r="H2" s="45" t="s">
         <v>1114</v>
+      </c>
+      <c r="I2" s="47">
+        <v>11384822337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>